<commit_message>
tentando usar lm na otimização dos pesos
</commit_message>
<xml_diff>
--- a/Peaks-dataset-article/media_ponderada/tabela_resultados_completa.xlsx
+++ b/Peaks-dataset-article/media_ponderada/tabela_resultados_completa.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K37"/>
+  <dimension ref="A1:J41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,45 +441,40 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>lr</t>
+          <t>n_epocas</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>n_epocas</t>
+          <t>mse_25</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>mse_25</t>
+          <t>mse_1000</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>mse_1000</t>
+          <t>r2_25</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>r2_25</t>
+          <t>r2_1000</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>r2_1000</t>
+          <t>var_25</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>var_25</t>
+          <t>bias_25</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>bias_25</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>covar_25</t>
         </is>
@@ -488,1332 +483,1360 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>[7.502851e-02, 7.891677e-02, 1.220961e-01, 8.495809e-02, 6.175034e-02, 9.317106e-02, 1.182250e-01, 1.354652e-01, 9.442332e-02, 1.359657e-01]</t>
+          <t>[1.414732e-01, 6.606663e-02, 7.822559e-02, 9.435053e-02, 1.276670e-01, 7.442410e-02, 9.314260e-02, 1.385867e-01, 6.479937e-02, 1.212643e-01]</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1e-06</v>
+        <v>1e-05</v>
       </c>
       <c r="C2" t="n">
-        <v>1e-05</v>
+        <v>500000</v>
       </c>
       <c r="D2" t="n">
-        <v>500000</v>
+        <v>0.02709016305486649</v>
       </c>
       <c r="E2" t="n">
-        <v>0.03249653665017917</v>
+        <v>0.6794575686799404</v>
       </c>
       <c r="F2" t="n">
-        <v>0.6668933836788108</v>
+        <v>0.9935450217011713</v>
       </c>
       <c r="G2" t="n">
-        <v>0.9922568041233581</v>
+        <v>0.8381004997304358</v>
       </c>
       <c r="H2" t="n">
-        <v>0.8410942632364178</v>
+        <v>0.06833543690345389</v>
       </c>
       <c r="I2" t="n">
-        <v>0.06864421605035986</v>
+        <v>0.01555916822650907</v>
       </c>
       <c r="J2" t="n">
-        <v>0.004673841822842597</v>
-      </c>
-      <c r="K2" t="n">
         <v>3.896305224157907</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>[1.349028e-01, 7.729080e-02, 1.180792e-01, 1.413648e-01, 7.961646e-02, 5.911507e-02, 5.933375e-02, 1.330312e-01, 1.160689e-01, 8.119696e-02]</t>
+          <t>[1.157707e-01, 7.689650e-02, 1.021228e-01, 8.278411e-02, 7.694917e-02, 1.025955e-01, 1.137894e-01, 1.182320e-01, 1.122955e-01, 9.856440e-02]</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1e-06</v>
+        <v>1e-05</v>
       </c>
       <c r="C3" t="n">
-        <v>1e-05</v>
+        <v>5000000</v>
       </c>
       <c r="D3" t="n">
-        <v>5000000</v>
+        <v>0.028891766738032</v>
       </c>
       <c r="E3" t="n">
-        <v>0.02809336124335244</v>
+        <v>0.6729760588036776</v>
       </c>
       <c r="F3" t="n">
-        <v>0.6776667783866756</v>
+        <v>0.9931157399484418</v>
       </c>
       <c r="G3" t="n">
-        <v>0.9933059820718053</v>
+        <v>0.8396448981716775</v>
       </c>
       <c r="H3" t="n">
-        <v>0.8385272048948664</v>
+        <v>0.06802503158224593</v>
       </c>
       <c r="I3" t="n">
-        <v>0.06849995384654156</v>
+        <v>0.01048027852874454</v>
       </c>
       <c r="J3" t="n">
-        <v>0.01194859806894259</v>
-      </c>
-      <c r="K3" t="n">
         <v>3.896305224157907</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>[1.112419e-01, 1.420950e-01, 9.709455e-02, 7.012772e-02, 1.472327e-01, 1.142142e-01, 1.028394e-01, 6.151295e-02, 6.669901e-02, 8.694271e-02]</t>
+          <t>[7.105069e-02, 7.602376e-02, 1.160450e-01, 6.269633e-02, 1.133646e-01, 1.165138e-01, 8.986475e-02, 9.706483e-02, 1.177914e-01, 1.395850e-01]</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1e-06</v>
+        <v>1e-05</v>
       </c>
       <c r="C4" t="n">
-        <v>1e-05</v>
+        <v>1000000</v>
       </c>
       <c r="D4" t="n">
-        <v>1000000</v>
+        <v>0.03089232143012372</v>
       </c>
       <c r="E4" t="n">
-        <v>0.01922749404325168</v>
+        <v>0.6678442556853932</v>
       </c>
       <c r="F4" t="n">
-        <v>0.7008562238995045</v>
+        <v>0.9926390526322039</v>
       </c>
       <c r="G4" t="n">
-        <v>0.9954185193888027</v>
+        <v>0.8408676917626684</v>
       </c>
       <c r="H4" t="n">
-        <v>0.8330016801040405</v>
+        <v>0.06849832093852411</v>
       </c>
       <c r="I4" t="n">
-        <v>0.06877617803120574</v>
+        <v>-0.0006874504728453723</v>
       </c>
       <c r="J4" t="n">
-        <v>0.001509308700459407</v>
-      </c>
-      <c r="K4" t="n">
         <v>3.896305224157907</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>[1.127636e-01, 8.472642e-02, 1.179376e-01, 8.246489e-02, 1.545599e-01, 1.498100e-01, 8.199804e-02, 6.720506e-02, 7.453132e-02, 7.400312e-02]</t>
+          <t>[9.062796e-02, 7.912693e-02, 8.303510e-02, 8.625625e-02, 1.446889e-01, 1.196652e-01, 1.259557e-01, 1.033115e-01, 7.234317e-02, 9.498926e-02]</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1e-06</v>
+        <v>1e-05</v>
       </c>
       <c r="C5" t="n">
-        <v>0.01</v>
+        <v>100</v>
       </c>
       <c r="D5" t="n">
-        <v>500000</v>
+        <v>0.02289153394301487</v>
       </c>
       <c r="E5" t="n">
-        <v>0.02081428494997335</v>
+        <v>0.6839374962038243</v>
       </c>
       <c r="F5" t="n">
-        <v>0.6922975267319471</v>
+        <v>0.9945454608549315</v>
       </c>
       <c r="G5" t="n">
-        <v>0.9950404227030454</v>
+        <v>0.837033033473831</v>
       </c>
       <c r="H5" t="n">
-        <v>0.8350410256912537</v>
+        <v>0.0680596928620549</v>
       </c>
       <c r="I5" t="n">
-        <v>0.06896509556367568</v>
+        <v>0.003032261523282021</v>
       </c>
       <c r="J5" t="n">
-        <v>-0.003948608928276854</v>
-      </c>
-      <c r="K5" t="n">
         <v>3.896305224157907</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>[9.264110e-02, 8.741962e-02, 1.030241e-01, 9.073466e-02, 7.464754e-02, 9.830046e-02, 1.562068e-01, 7.887357e-02, 1.033128e-01, 1.148393e-01]</t>
+          <t>[9.128113e-02, 1.066367e-01, 1.220262e-01, 1.135682e-01, 1.246721e-01, 1.086222e-01, 7.797398e-02, 7.183605e-02, 1.056874e-01, 7.769604e-02]</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1e-06</v>
+        <v>1e-05</v>
       </c>
       <c r="C6" t="n">
-        <v>0.01</v>
+        <v>5000</v>
       </c>
       <c r="D6" t="n">
-        <v>5000000</v>
+        <v>0.02191097352003641</v>
       </c>
       <c r="E6" t="n">
-        <v>0.02625988191840158</v>
+        <v>0.687772283781353</v>
       </c>
       <c r="F6" t="n">
-        <v>0.6795612782644023</v>
+        <v>0.9947791064124792</v>
       </c>
       <c r="G6" t="n">
-        <v>0.9937428590750902</v>
+        <v>0.8361192895977445</v>
       </c>
       <c r="H6" t="n">
-        <v>0.8380757880623766</v>
+        <v>0.06817642575039141</v>
       </c>
       <c r="I6" t="n">
-        <v>0.06797925116733919</v>
+        <v>-0.002488828414728302</v>
       </c>
       <c r="J6" t="n">
-        <v>0.007513762662632904</v>
-      </c>
-      <c r="K6" t="n">
         <v>3.896305224157907</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>[7.822184e-02, 8.817460e-02, 7.699271e-02, 1.654094e-01, 7.223314e-02, 1.380720e-01, 7.432468e-02, 6.446405e-02, 1.504887e-01, 9.161890e-02]</t>
+          <t>[9.348313e-02, 1.005888e-01, 1.309916e-01, 7.619396e-02, 6.306213e-02, 1.198581e-01, 1.236627e-01, 1.196893e-01, 5.000067e-02, 1.224696e-01]</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1e-06</v>
+        <v>5e-06</v>
       </c>
       <c r="C7" t="n">
-        <v>0.01</v>
+        <v>500000</v>
       </c>
       <c r="D7" t="n">
-        <v>1000000</v>
+        <v>0.0270494714875424</v>
       </c>
       <c r="E7" t="n">
-        <v>0.02436043624761087</v>
+        <v>0.6784051020393806</v>
       </c>
       <c r="F7" t="n">
-        <v>0.6676452870218474</v>
+        <v>0.9935547175890658</v>
       </c>
       <c r="G7" t="n">
-        <v>0.9941954543791467</v>
+        <v>0.8383512789269765</v>
       </c>
       <c r="H7" t="n">
-        <v>0.8409151015328766</v>
+        <v>0.06801738344942541</v>
       </c>
       <c r="I7" t="n">
-        <v>0.0682637969488487</v>
+        <v>0.002125913588287474</v>
       </c>
       <c r="J7" t="n">
-        <v>0.003296989373916506</v>
-      </c>
-      <c r="K7" t="n">
         <v>3.896305224157907</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>[7.016232e-02, 1.587711e-01, 8.405561e-02, 8.659333e-02, 6.299641e-02, 8.589770e-02, 1.482177e-01, 1.310295e-01, 1.089168e-01, 6.335954e-02]</t>
+          <t>[1.224746e-01, 7.684429e-02, 7.236259e-02, 6.671564e-02, 8.560880e-02, 1.188436e-01, 1.476652e-01, 6.372245e-02, 1.423906e-01, 1.033722e-01]</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1e-06</v>
+        <v>5e-06</v>
       </c>
       <c r="C8" t="n">
-        <v>0.001</v>
+        <v>5000000</v>
       </c>
       <c r="D8" t="n">
-        <v>500000</v>
+        <v>0.02732306518816444</v>
       </c>
       <c r="E8" t="n">
-        <v>0.02531264804935399</v>
+        <v>0.6756128814639886</v>
       </c>
       <c r="F8" t="n">
-        <v>0.6853476979482991</v>
+        <v>0.9934895263461547</v>
       </c>
       <c r="G8" t="n">
-        <v>0.9939685636622584</v>
+        <v>0.839016602468337</v>
       </c>
       <c r="H8" t="n">
-        <v>0.8366970140250325</v>
+        <v>0.06821700807711517</v>
       </c>
       <c r="I8" t="n">
-        <v>0.06825897048573011</v>
+        <v>0.01409261524076718</v>
       </c>
       <c r="J8" t="n">
-        <v>0.00793848574486764</v>
-      </c>
-      <c r="K8" t="n">
         <v>3.896305224157907</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>[1.397206e-01, 6.697167e-02, 8.989919e-02, 8.222334e-02, 9.698563e-02, 1.052449e-01, 1.169575e-01, 1.404536e-01, 7.609047e-02, 8.545314e-02]</t>
+          <t>[1.267061e-01, 1.055798e-01, 1.199531e-01, 6.411445e-02, 1.430739e-01, 6.831253e-02, 8.898214e-02, 9.668674e-02, 7.604176e-02, 1.105495e-01]</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1e-06</v>
+        <v>5e-06</v>
       </c>
       <c r="C9" t="n">
-        <v>0.001</v>
+        <v>1000000</v>
       </c>
       <c r="D9" t="n">
-        <v>5000000</v>
+        <v>0.02492358083058264</v>
       </c>
       <c r="E9" t="n">
-        <v>0.02682162791044481</v>
+        <v>0.6922855032691175</v>
       </c>
       <c r="F9" t="n">
-        <v>0.6785079235741843</v>
+        <v>0.994061269654794</v>
       </c>
       <c r="G9" t="n">
-        <v>0.9936090076035893</v>
+        <v>0.8350438906127932</v>
       </c>
       <c r="H9" t="n">
-        <v>0.8383267788612343</v>
+        <v>0.06834988219559543</v>
       </c>
       <c r="I9" t="n">
-        <v>0.06812015038815598</v>
+        <v>0.006151664743014065</v>
       </c>
       <c r="J9" t="n">
-        <v>0.01369891330168702</v>
-      </c>
-      <c r="K9" t="n">
         <v>3.896305224157907</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>[6.178473e-02, 9.538793e-02, 7.951448e-02, 1.005421e-01, 1.264809e-01, 9.514446e-02, 1.508431e-01, 1.168877e-01, 9.435074e-02, 7.906385e-02]</t>
+          <t>[1.003278e-01, 1.031346e-01, 8.078505e-02, 1.407201e-01, 8.058368e-02, 1.357591e-01, 9.296866e-02, 9.117644e-02, 9.142974e-02, 8.311494e-02]</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1e-06</v>
+        <v>5e-06</v>
       </c>
       <c r="C10" t="n">
-        <v>0.001</v>
+        <v>100</v>
       </c>
       <c r="D10" t="n">
-        <v>1000000</v>
+        <v>0.0219478243212043</v>
       </c>
       <c r="E10" t="n">
-        <v>0.0238619347823744</v>
+        <v>0.6787644591768671</v>
       </c>
       <c r="F10" t="n">
-        <v>0.6836078210946339</v>
+        <v>0.994770325693022</v>
       </c>
       <c r="G10" t="n">
-        <v>0.9943142360983087</v>
+        <v>0.8382656521804963</v>
       </c>
       <c r="H10" t="n">
-        <v>0.8371115876586536</v>
+        <v>0.06814268724563317</v>
       </c>
       <c r="I10" t="n">
-        <v>0.06820211886195122</v>
+        <v>0.005235265801462614</v>
       </c>
       <c r="J10" t="n">
-        <v>0.003260995837935381</v>
-      </c>
-      <c r="K10" t="n">
         <v>3.896305224157907</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>[9.166573e-02, 8.945216e-02, 1.362759e-01, 8.206687e-02, 6.282444e-02, 1.097558e-01, 1.113999e-01, 1.297131e-01, 8.760526e-02, 9.924085e-02]</t>
+          <t>[8.149546e-02, 1.476992e-01, 1.163065e-01, 5.774675e-02, 1.220063e-01, 7.458462e-02, 7.065140e-02, 8.667124e-02, 9.676358e-02, 1.460751e-01]</t>
         </is>
       </c>
       <c r="B11" t="n">
         <v>5e-06</v>
       </c>
       <c r="C11" t="n">
-        <v>1e-05</v>
+        <v>5000</v>
       </c>
       <c r="D11" t="n">
-        <v>500000</v>
+        <v>0.02709791853763094</v>
       </c>
       <c r="E11" t="n">
-        <v>0.02899663014264296</v>
+        <v>0.6833474869533233</v>
       </c>
       <c r="F11" t="n">
-        <v>0.6744786012761399</v>
+        <v>0.9935431737435625</v>
       </c>
       <c r="G11" t="n">
-        <v>0.993090753350918</v>
+        <v>0.8371736194459558</v>
       </c>
       <c r="H11" t="n">
-        <v>0.8392868759983458</v>
+        <v>0.06811084607633013</v>
       </c>
       <c r="I11" t="n">
-        <v>0.06810795162428113</v>
+        <v>0.001175261467824289</v>
       </c>
       <c r="J11" t="n">
-        <v>0.002421206390047994</v>
-      </c>
-      <c r="K11" t="n">
         <v>3.896305224157907</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>[9.884183e-02, 7.993027e-02, 1.515485e-01, 7.394134e-02, 7.716098e-02, 7.064907e-02, 7.803023e-02, 1.318418e-01, 1.452408e-01, 9.281521e-02]</t>
+          <t>[8.008492e-02, 1.079585e-01, 1.404401e-01, 1.281148e-01, 7.194693e-02, 9.649869e-02, 7.296768e-02, 7.832660e-02, 1.406008e-01, 8.306096e-02]</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>5e-06</v>
+        <v>1e-07</v>
       </c>
       <c r="C12" t="n">
-        <v>1e-05</v>
+        <v>500000</v>
       </c>
       <c r="D12" t="n">
-        <v>5000000</v>
+        <v>0.02605515849496684</v>
       </c>
       <c r="E12" t="n">
-        <v>0.03370949173075977</v>
+        <v>0.6778786064209741</v>
       </c>
       <c r="F12" t="n">
-        <v>0.6718071694404354</v>
+        <v>0.9937916400755167</v>
       </c>
       <c r="G12" t="n">
-        <v>0.9919677841308707</v>
+        <v>0.8384767310250077</v>
       </c>
       <c r="H12" t="n">
-        <v>0.839923418291995</v>
+        <v>0.0680936546968646</v>
       </c>
       <c r="I12" t="n">
-        <v>0.06886617013882393</v>
+        <v>-0.00164042032821128</v>
       </c>
       <c r="J12" t="n">
-        <v>0.004128823845848939</v>
-      </c>
-      <c r="K12" t="n">
         <v>3.896305224157907</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>[7.353196e-02, 1.178449e-01, 6.681582e-02, 1.153669e-01, 7.647605e-02, 1.299230e-01, 8.494118e-02, 7.072035e-02, 1.665096e-01, 9.787030e-02]</t>
+          <t>[1.284914e-01, 8.011043e-02, 1.054328e-01, 1.132545e-01, 9.408262e-02, 1.329785e-01, 9.758160e-02, 7.878056e-02, 1.046580e-01, 6.462959e-02]</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>5e-06</v>
+        <v>1e-07</v>
       </c>
       <c r="C13" t="n">
-        <v>1e-05</v>
+        <v>5000000</v>
       </c>
       <c r="D13" t="n">
-        <v>1000000</v>
+        <v>0.02254146723953925</v>
       </c>
       <c r="E13" t="n">
-        <v>0.02664704329957533</v>
+        <v>0.6835774535683824</v>
       </c>
       <c r="F13" t="n">
-        <v>0.6678091663976028</v>
+        <v>0.9946288738993454</v>
       </c>
       <c r="G13" t="n">
-        <v>0.9936506072009114</v>
+        <v>0.8371188235590999</v>
       </c>
       <c r="H13" t="n">
-        <v>0.8408760527529935</v>
+        <v>0.06819125370549139</v>
       </c>
       <c r="I13" t="n">
-        <v>0.06829722663943595</v>
+        <v>0.005658908425951831</v>
       </c>
       <c r="J13" t="n">
-        <v>0.005600879727250387</v>
-      </c>
-      <c r="K13" t="n">
         <v>3.896305224157907</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>[9.324632e-02, 1.125555e-01, 1.336425e-01, 1.267796e-01, 9.477851e-02, 1.021174e-01, 1.109665e-01, 8.293596e-02, 8.665828e-02, 5.631932e-02]</t>
+          <t>[1.407752e-01, 7.454336e-02, 1.208936e-01, 9.387800e-02, 6.649483e-02, 1.255335e-01, 6.764744e-02, 8.320815e-02, 1.162015e-01, 1.108246e-01]</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>5e-06</v>
+        <v>1e-07</v>
       </c>
       <c r="C14" t="n">
-        <v>0.01</v>
+        <v>1000000</v>
       </c>
       <c r="D14" t="n">
-        <v>500000</v>
+        <v>0.0282491126972747</v>
       </c>
       <c r="E14" t="n">
-        <v>0.02072855954797621</v>
+        <v>0.6726766859182531</v>
       </c>
       <c r="F14" t="n">
-        <v>0.6937000000629139</v>
+        <v>0.9932688699934084</v>
       </c>
       <c r="G14" t="n">
-        <v>0.9950608491437586</v>
+        <v>0.8397162320161715</v>
       </c>
       <c r="H14" t="n">
-        <v>0.8347068477500674</v>
+        <v>0.06823808454671165</v>
       </c>
       <c r="I14" t="n">
-        <v>0.06836380447501081</v>
+        <v>0.008384456384646162</v>
       </c>
       <c r="J14" t="n">
-        <v>-0.00149190299712502</v>
-      </c>
-      <c r="K14" t="n">
         <v>3.896305224157907</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>[9.215754e-02, 7.293370e-02, 8.330952e-02, 1.471232e-01, 9.181012e-02, 9.480526e-02, 8.140153e-02, 1.601613e-01, 8.870397e-02, 8.759382e-02]</t>
+          <t>[1.043152e-01, 7.142242e-02, 8.646363e-02, 1.535501e-01, 1.272106e-01, 9.680646e-02, 6.000972e-02, 6.867127e-02, 1.049370e-01, 1.266136e-01]</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>5e-06</v>
+        <v>1e-07</v>
       </c>
       <c r="C15" t="n">
-        <v>0.01</v>
+        <v>100</v>
       </c>
       <c r="D15" t="n">
-        <v>5000000</v>
+        <v>0.02331409315314314</v>
       </c>
       <c r="E15" t="n">
-        <v>0.02679163214176446</v>
+        <v>0.676758834764601</v>
       </c>
       <c r="F15" t="n">
-        <v>0.6695769558264446</v>
+        <v>0.9944447744719878</v>
       </c>
       <c r="G15" t="n">
-        <v>0.993616154922544</v>
+        <v>0.8387435474973521</v>
       </c>
       <c r="H15" t="n">
-        <v>0.8404548281787094</v>
+        <v>0.06797881427960573</v>
       </c>
       <c r="I15" t="n">
-        <v>0.06800623967696366</v>
+        <v>0.005122792586947488</v>
       </c>
       <c r="J15" t="n">
-        <v>0.008103153785920024</v>
-      </c>
-      <c r="K15" t="n">
         <v>3.896305224157907</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>[1.432924e-01, 1.532407e-01, 6.170186e-02, 7.218489e-02, 6.314956e-02, 1.353372e-01, 7.999278e-02, 1.332678e-01, 1.001974e-01, 5.763534e-02]</t>
+          <t>[6.524672e-02, 1.077605e-01, 1.171564e-01, 7.604721e-02, 1.268429e-01, 9.545890e-02, 8.143324e-02, 1.200365e-01, 8.925063e-02, 1.207670e-01]</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>5e-06</v>
+        <v>1e-07</v>
       </c>
       <c r="C16" t="n">
-        <v>0.01</v>
+        <v>5000</v>
       </c>
       <c r="D16" t="n">
-        <v>1000000</v>
+        <v>0.02762833804245024</v>
       </c>
       <c r="E16" t="n">
-        <v>0.0249174563350629</v>
+        <v>0.6770103052876563</v>
       </c>
       <c r="F16" t="n">
-        <v>0.6820476756105148</v>
+        <v>0.993416786671401</v>
       </c>
       <c r="G16" t="n">
-        <v>0.9940627289847209</v>
+        <v>0.8386836277114936</v>
       </c>
       <c r="H16" t="n">
-        <v>0.8374833353377874</v>
+        <v>0.06820249916565763</v>
       </c>
       <c r="I16" t="n">
-        <v>0.06853795508385262</v>
+        <v>-0.002183089555671125</v>
       </c>
       <c r="J16" t="n">
-        <v>0.01551354413499067</v>
-      </c>
-      <c r="K16" t="n">
         <v>3.896305224157907</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>[9.813736e-02, 1.190849e-01, 8.841580e-02, 1.510060e-01, 1.049567e-01, 1.090371e-01, 6.144301e-02, 8.714099e-02, 6.428301e-02, 1.164951e-01]</t>
+          <t>[6.132993e-02, 1.027096e-01, 8.911299e-02, 1.253380e-01, 1.346551e-01, 8.236684e-02, 9.088614e-02, 1.147861e-01, 5.915458e-02, 1.396607e-01]</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>5e-06</v>
+        <v>0.001</v>
       </c>
       <c r="C17" t="n">
-        <v>0.001</v>
+        <v>500000</v>
       </c>
       <c r="D17" t="n">
-        <v>500000</v>
+        <v>0.0242637086903871</v>
       </c>
       <c r="E17" t="n">
-        <v>0.0208832135056408</v>
+        <v>0.6798609583916478</v>
       </c>
       <c r="F17" t="n">
-        <v>0.6833855266062043</v>
+        <v>0.9942185023867026</v>
       </c>
       <c r="G17" t="n">
-        <v>0.995023998574106</v>
+        <v>0.8380043810090472</v>
       </c>
       <c r="H17" t="n">
-        <v>0.8371645554497981</v>
+        <v>0.06811634302254629</v>
       </c>
       <c r="I17" t="n">
-        <v>0.06810409196696421</v>
+        <v>0.0006547790795843355</v>
       </c>
       <c r="J17" t="n">
-        <v>0.003138615058201056</v>
-      </c>
-      <c r="K17" t="n">
         <v>3.896305224157907</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>[9.211974e-02, 8.706166e-02, 1.486199e-01, 8.239054e-02, 8.759033e-02, 9.200453e-02, 8.921192e-02, 7.516377e-02, 7.888624e-02, 1.669514e-01]</t>
+          <t>[1.486014e-01, 1.008728e-01, 7.313144e-02, 8.488319e-02, 8.063704e-02, 1.373197e-01, 1.125181e-01, 6.669272e-02, 1.239418e-01, 7.140170e-02]</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>5e-06</v>
+        <v>0.001</v>
       </c>
       <c r="C18" t="n">
-        <v>0.001</v>
+        <v>5000000</v>
       </c>
       <c r="D18" t="n">
-        <v>5000000</v>
+        <v>0.02369904798512891</v>
       </c>
       <c r="E18" t="n">
-        <v>0.02890416677070095</v>
+        <v>0.6833433033330657</v>
       </c>
       <c r="F18" t="n">
-        <v>0.6765718344233983</v>
+        <v>0.9943530483689936</v>
       </c>
       <c r="G18" t="n">
-        <v>0.993112785298755</v>
+        <v>0.8371746163088363</v>
       </c>
       <c r="H18" t="n">
-        <v>0.8387881054847622</v>
+        <v>0.06854911066150077</v>
       </c>
       <c r="I18" t="n">
-        <v>0.06818915872098098</v>
+        <v>0.01397606594030155</v>
       </c>
       <c r="J18" t="n">
-        <v>-0.000232686778698763</v>
-      </c>
-      <c r="K18" t="n">
         <v>3.896305224157907</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>[1.007285e-01, 6.057683e-02, 7.069949e-02, 1.379073e-01, 6.238451e-02, 9.223319e-02, 1.544429e-01, 6.826431e-02, 1.267687e-01, 1.259942e-01]</t>
+          <t>[6.303997e-02, 5.856388e-02, 1.508881e-01, 7.333019e-02, 6.886351e-02, 1.456787e-01, 1.500059e-01, 8.423624e-02, 1.474550e-01, 5.793856e-02]</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>5e-06</v>
+        <v>0.001</v>
       </c>
       <c r="C19" t="n">
-        <v>0.001</v>
+        <v>1000000</v>
       </c>
       <c r="D19" t="n">
-        <v>1000000</v>
+        <v>0.0292488932995395</v>
       </c>
       <c r="E19" t="n">
-        <v>0.02693301543669547</v>
+        <v>0.673947567905427</v>
       </c>
       <c r="F19" t="n">
-        <v>0.6724839247050596</v>
+        <v>0.9930306446981918</v>
       </c>
       <c r="G19" t="n">
-        <v>0.9935824664541967</v>
+        <v>0.8394134093409826</v>
       </c>
       <c r="H19" t="n">
-        <v>0.8397621626901768</v>
+        <v>0.06891021490464039</v>
       </c>
       <c r="I19" t="n">
-        <v>0.06833281034700545</v>
+        <v>-0.00552569804865882</v>
       </c>
       <c r="J19" t="n">
-        <v>0.01430694700245879</v>
-      </c>
-      <c r="K19" t="n">
         <v>3.896305224157907</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>[1.342220e-01, 6.265515e-02, 6.488497e-02, 1.454803e-01, 7.272935e-02, 1.227229e-01, 1.300710e-01, 8.628837e-02, 6.000798e-02, 1.209380e-01]</t>
+          <t>[9.178400e-02, 9.201244e-02, 1.099894e-01, 1.401071e-01, 8.021298e-02, 1.083806e-01, 7.343981e-02, 8.179264e-02, 7.362604e-02, 1.486550e-01]</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>1e-05</v>
+        <v>0.001</v>
       </c>
       <c r="C20" t="n">
-        <v>1e-05</v>
+        <v>100</v>
       </c>
       <c r="D20" t="n">
-        <v>500000</v>
+        <v>0.02498153257591994</v>
       </c>
       <c r="E20" t="n">
-        <v>0.02298226682185679</v>
+        <v>0.6739254518364557</v>
       </c>
       <c r="F20" t="n">
-        <v>0.6788313503090706</v>
+        <v>0.9940474610535769</v>
       </c>
       <c r="G20" t="n">
-        <v>0.99452384124479</v>
+        <v>0.8394186791042164</v>
       </c>
       <c r="H20" t="n">
-        <v>0.8382497135238747</v>
+        <v>0.06787379837476015</v>
       </c>
       <c r="I20" t="n">
-        <v>0.06844436883298295</v>
+        <v>0.0024986182646757</v>
       </c>
       <c r="J20" t="n">
-        <v>0.01478842553355655</v>
-      </c>
-      <c r="K20" t="n">
         <v>3.896305224157907</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>[1.209816e-01, 1.494090e-01, 6.673236e-02, 6.183597e-02, 1.056339e-01, 1.010695e-01, 6.234351e-02, 9.629710e-02, 8.821994e-02, 1.474771e-01]</t>
+          <t>[7.505583e-02, 1.645075e-01, 1.289852e-01, 8.248829e-02, 9.198837e-02, 6.830267e-02, 1.609420e-01, 6.858245e-02, 9.045190e-02, 6.869583e-02]</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>1e-05</v>
+        <v>0.001</v>
       </c>
       <c r="C21" t="n">
-        <v>1e-05</v>
+        <v>5000</v>
       </c>
       <c r="D21" t="n">
-        <v>5000000</v>
+        <v>0.02115372709946156</v>
       </c>
       <c r="E21" t="n">
-        <v>0.02636332996237335</v>
+        <v>0.7043350002041726</v>
       </c>
       <c r="F21" t="n">
-        <v>0.6789563386499357</v>
+        <v>0.9949595412515674</v>
       </c>
       <c r="G21" t="n">
-        <v>0.9937182097262641</v>
+        <v>0.8321727657299324</v>
       </c>
       <c r="H21" t="n">
-        <v>0.838219931605388</v>
+        <v>0.06871270290425113</v>
       </c>
       <c r="I21" t="n">
-        <v>0.06809388729773436</v>
+        <v>0.0004348634071801749</v>
       </c>
       <c r="J21" t="n">
-        <v>0.01200990182792289</v>
-      </c>
-      <c r="K21" t="n">
         <v>3.896305224157907</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>[1.075011e-01, 9.999090e-02, 1.045602e-01, 7.202749e-02, 1.191366e-01, 5.933006e-02, 1.099184e-01, 1.191574e-01, 1.010665e-01, 1.073113e-01]</t>
+          <t>[1.600129e-01, 8.203050e-02, 7.130042e-02, 9.996204e-02, 6.671480e-02, 1.375604e-01, 1.338790e-01, 6.639878e-02, 8.645209e-02, 9.568908e-02]</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>1e-05</v>
+        <v>0.1</v>
       </c>
       <c r="C22" t="n">
-        <v>1e-05</v>
+        <v>500000</v>
       </c>
       <c r="D22" t="n">
-        <v>1000000</v>
+        <v>0.02346574234764692</v>
       </c>
       <c r="E22" t="n">
-        <v>0.0276412986931742</v>
+        <v>0.6844594014729504</v>
       </c>
       <c r="F22" t="n">
-        <v>0.683316397208938</v>
+        <v>0.9944086398700079</v>
       </c>
       <c r="G22" t="n">
-        <v>0.9934136984390048</v>
+        <v>0.8369086751530843</v>
       </c>
       <c r="H22" t="n">
-        <v>0.8371810274347862</v>
+        <v>0.06891276198833364</v>
       </c>
       <c r="I22" t="n">
-        <v>0.06808138948549824</v>
+        <v>0.01678365364259505</v>
       </c>
       <c r="J22" t="n">
-        <v>0.009348957228024722</v>
-      </c>
-      <c r="K22" t="n">
         <v>3.896305224157907</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>[1.382908e-01, 1.462981e-01, 7.014243e-02, 1.637330e-01, 7.320510e-02, 1.025153e-01, 7.465755e-02, 7.435987e-02, 7.477477e-02, 8.202318e-02]</t>
+          <t>[1.163836e-01, 8.355706e-02, 8.570179e-02, 7.571281e-02, 6.793821e-02, 1.225014e-01, 7.951571e-02, 1.609166e-01, 8.754532e-02, 1.202276e-01]</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>1e-05</v>
+        <v>0.1</v>
       </c>
       <c r="C23" t="n">
-        <v>0.01</v>
+        <v>5000000</v>
       </c>
       <c r="D23" t="n">
-        <v>500000</v>
+        <v>0.03180962599577317</v>
       </c>
       <c r="E23" t="n">
-        <v>0.01888490631659547</v>
+        <v>0.6633767336178265</v>
       </c>
       <c r="F23" t="n">
-        <v>0.6946119137501953</v>
+        <v>0.9924204795268042</v>
       </c>
       <c r="G23" t="n">
-        <v>0.9955001503607732</v>
+        <v>0.8419322020772528</v>
       </c>
       <c r="H23" t="n">
-        <v>0.8344895591700805</v>
+        <v>0.06851037714343074</v>
       </c>
       <c r="I23" t="n">
-        <v>0.06907371673613494</v>
+        <v>0.01192592532725194</v>
       </c>
       <c r="J23" t="n">
-        <v>0.01246622724469235</v>
-      </c>
-      <c r="K23" t="n">
         <v>3.896305224157907</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>[1.009450e-01, 1.090151e-01, 1.076731e-01, 1.056828e-01, 1.325718e-01, 5.348190e-02, 9.374127e-02, 1.287242e-01, 5.782677e-02, 1.103381e-01]</t>
+          <t>[1.583428e-01, 1.346849e-01, 7.728409e-02, 8.628064e-02, 6.906470e-02, 1.035953e-01, 1.492255e-01, 7.289429e-02, 7.819758e-02, 7.043031e-02]</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>1e-05</v>
+        <v>0.1</v>
       </c>
       <c r="C24" t="n">
-        <v>0.01</v>
+        <v>1000000</v>
       </c>
       <c r="D24" t="n">
-        <v>5000000</v>
+        <v>0.02134449773892111</v>
       </c>
       <c r="E24" t="n">
-        <v>0.02426483811992609</v>
+        <v>0.70028995133752</v>
       </c>
       <c r="F24" t="n">
-        <v>0.6894998886787458</v>
+        <v>0.99491408488664</v>
       </c>
       <c r="G24" t="n">
-        <v>0.9942182332689734</v>
+        <v>0.83313661015564</v>
       </c>
       <c r="H24" t="n">
-        <v>0.8357076400960772</v>
+        <v>0.06925395944162051</v>
       </c>
       <c r="I24" t="n">
-        <v>0.06814581512539536</v>
+        <v>0.01744320707388072</v>
       </c>
       <c r="J24" t="n">
-        <v>0.00590744254726908</v>
-      </c>
-      <c r="K24" t="n">
         <v>3.896305224157907</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>[9.642991e-02, 9.174332e-02, 1.416938e-01, 9.630423e-02, 1.084027e-01, 6.635923e-02, 1.004944e-01, 9.932124e-02, 1.119408e-01, 8.731035e-02]</t>
+          <t>[1.033102e-01, 9.201891e-02, 7.747568e-02, 9.740352e-02, 1.483136e-01, 7.552981e-02, 7.312296e-02, 7.534967e-02, 8.843565e-02, 1.690399e-01]</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>1e-05</v>
+        <v>0.1</v>
       </c>
       <c r="C25" t="n">
-        <v>0.01</v>
+        <v>100</v>
       </c>
       <c r="D25" t="n">
-        <v>1000000</v>
+        <v>0.02583788310776396</v>
       </c>
       <c r="E25" t="n">
-        <v>0.02644158846768443</v>
+        <v>0.6784871307304994</v>
       </c>
       <c r="F25" t="n">
-        <v>0.6855046209488597</v>
+        <v>0.9938434119274034</v>
       </c>
       <c r="G25" t="n">
-        <v>0.9936995624795695</v>
+        <v>0.8383317333295587</v>
       </c>
       <c r="H25" t="n">
-        <v>0.8366596227933462</v>
+        <v>0.06802148477423973</v>
       </c>
       <c r="I25" t="n">
-        <v>0.06814911472310906</v>
+        <v>0.00796157579851613</v>
       </c>
       <c r="J25" t="n">
-        <v>0.001848754814770939</v>
-      </c>
-      <c r="K25" t="n">
         <v>3.896305224157907</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>[1.246794e-01, 1.440836e-01, 9.657973e-02, 9.475866e-02, 1.565117e-01, 6.874437e-02, 8.583385e-02, 9.569267e-02, 5.867957e-02, 7.443642e-02]</t>
+          <t>[1.034338e-01, 1.156735e-01, 1.212358e-01, 7.220086e-02, 1.114912e-01, 1.255303e-01, 5.998913e-02, 9.325841e-02, 1.189630e-01, 7.822393e-02]</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>1e-05</v>
+        <v>0.1</v>
       </c>
       <c r="C26" t="n">
-        <v>0.001</v>
+        <v>5000</v>
       </c>
       <c r="D26" t="n">
-        <v>500000</v>
+        <v>0.02539569636000464</v>
       </c>
       <c r="E26" t="n">
-        <v>0.0194733619243127</v>
+        <v>0.6806005771304227</v>
       </c>
       <c r="F26" t="n">
-        <v>0.7053341388807919</v>
+        <v>0.9939487751123733</v>
       </c>
       <c r="G26" t="n">
-        <v>0.9953599345868798</v>
+        <v>0.8378281464511921</v>
       </c>
       <c r="H26" t="n">
-        <v>0.8319346933912006</v>
+        <v>0.06805746833765766</v>
       </c>
       <c r="I26" t="n">
-        <v>0.06905216123278551</v>
+        <v>-0.0002794988073275151</v>
       </c>
       <c r="J26" t="n">
-        <v>0.00591690100632423</v>
-      </c>
-      <c r="K26" t="n">
         <v>3.896305224157907</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>[9.772351e-02, 9.324025e-02, 8.500804e-02, 6.203091e-02, 6.502396e-02, 1.539981e-01, 1.217993e-01, 1.266511e-01, 1.048189e-01, 8.970593e-02]</t>
+          <t>[9.774661e-02, 7.794409e-02, 7.593677e-02, 1.526948e-01, 7.437458e-02, 7.399876e-02, 1.364944e-01, 8.302367e-02, 1.176570e-01, 1.101293e-01]</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>1e-05</v>
+        <v>0.01</v>
       </c>
       <c r="C27" t="n">
-        <v>0.001</v>
+        <v>500000</v>
       </c>
       <c r="D27" t="n">
-        <v>5000000</v>
+        <v>0.02514383758405269</v>
       </c>
       <c r="E27" t="n">
-        <v>0.02893135180652828</v>
+        <v>0.6780295958573134</v>
       </c>
       <c r="F27" t="n">
-        <v>0.6684814984712445</v>
+        <v>0.9940087874101896</v>
       </c>
       <c r="G27" t="n">
-        <v>0.9931063077144023</v>
+        <v>0.8384407536286019</v>
       </c>
       <c r="H27" t="n">
-        <v>0.8407158510983865</v>
+        <v>0.06817604667387915</v>
       </c>
       <c r="I27" t="n">
-        <v>0.06848360222056388</v>
+        <v>0.01277391847438972</v>
       </c>
       <c r="J27" t="n">
-        <v>0.007320345583173306</v>
-      </c>
-      <c r="K27" t="n">
         <v>3.896305224157907</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>[8.084298e-02, 6.421661e-02, 1.212379e-01, 1.385674e-01, 7.804759e-02, 7.822415e-02, 1.128052e-01, 8.518262e-02, 1.095353e-01, 1.313402e-01]</t>
+          <t>[9.732225e-02, 9.469433e-02, 8.192600e-02, 6.939663e-02, 1.595812e-01, 7.170098e-02, 8.320215e-02, 1.502524e-01, 1.128062e-01, 7.911789e-02]</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>1e-05</v>
+        <v>0.01</v>
       </c>
       <c r="C28" t="n">
-        <v>0.001</v>
+        <v>5000000</v>
       </c>
       <c r="D28" t="n">
-        <v>1000000</v>
+        <v>0.02739462539123538</v>
       </c>
       <c r="E28" t="n">
-        <v>0.02771355823113816</v>
+        <v>0.6799795207320314</v>
       </c>
       <c r="F28" t="n">
-        <v>0.6731301106102752</v>
+        <v>0.9934724751546595</v>
       </c>
       <c r="G28" t="n">
-        <v>0.9933964806116888</v>
+        <v>0.837976130262358</v>
       </c>
       <c r="H28" t="n">
-        <v>0.8396081910811197</v>
+        <v>0.06810344825453458</v>
       </c>
       <c r="I28" t="n">
-        <v>0.06810982023043255</v>
+        <v>0.007621554600512712</v>
       </c>
       <c r="J28" t="n">
-        <v>0.0039366723361217</v>
-      </c>
-      <c r="K28" t="n">
         <v>3.896305224157907</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>[1.112902e-01, 7.244882e-02, 1.508716e-01, 1.126127e-01, 5.742278e-02, 6.870735e-02, 1.322370e-01, 8.883105e-02, 6.701565e-02, 1.385628e-01]</t>
+          <t>[7.613931e-02, 1.195353e-01, 1.029382e-01, 1.114420e-01, 1.049578e-01, 6.653746e-02, 1.011093e-01, 1.036435e-01, 1.219099e-01, 9.178720e-02]</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>0.001</v>
+        <v>0.01</v>
       </c>
       <c r="C29" t="n">
-        <v>1e-05</v>
+        <v>1000000</v>
       </c>
       <c r="D29" t="n">
-        <v>500000</v>
+        <v>0.02554090188377162</v>
       </c>
       <c r="E29" t="n">
-        <v>0.02760032068502105</v>
+        <v>0.682353653584773</v>
       </c>
       <c r="F29" t="n">
-        <v>0.6827110196730387</v>
+        <v>0.9939141758926164</v>
       </c>
       <c r="G29" t="n">
-        <v>0.9934234625793248</v>
+        <v>0.8374104276487582</v>
       </c>
       <c r="H29" t="n">
-        <v>0.8373252753246536</v>
+        <v>0.06801316676492056</v>
       </c>
       <c r="I29" t="n">
-        <v>0.06824826056671436</v>
+        <v>0.004284302533106272</v>
       </c>
       <c r="J29" t="n">
-        <v>0.006062838744853467</v>
-      </c>
-      <c r="K29" t="n">
         <v>3.896305224157907</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>[8.094721e-02, 7.785576e-02, 9.437270e-02, 6.005929e-02, 1.404789e-01, 1.336603e-01, 1.252190e-01, 1.294769e-01, 7.009652e-02, 8.783338e-02]</t>
+          <t>[1.099324e-01, 1.203495e-01, 8.223149e-02, 5.797903e-02, 1.289652e-01, 8.974434e-02, 6.814930e-02, 1.471666e-01, 5.967682e-02, 1.358052e-01]</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>0.001</v>
+        <v>0.01</v>
       </c>
       <c r="C30" t="n">
-        <v>1e-05</v>
+        <v>100</v>
       </c>
       <c r="D30" t="n">
-        <v>5000000</v>
+        <v>0.0276960923908505</v>
       </c>
       <c r="E30" t="n">
-        <v>0.02530599672789549</v>
+        <v>0.6775593907107031</v>
       </c>
       <c r="F30" t="n">
-        <v>0.6796349587187422</v>
+        <v>0.9934006423297191</v>
       </c>
       <c r="G30" t="n">
-        <v>0.9939701485229913</v>
+        <v>0.8385527929696432</v>
       </c>
       <c r="H30" t="n">
-        <v>0.8380582316625554</v>
+        <v>0.06803219554944485</v>
       </c>
       <c r="I30" t="n">
-        <v>0.06819143253262921</v>
+        <v>0.008956850724787331</v>
       </c>
       <c r="J30" t="n">
-        <v>0.0002888855528642087</v>
-      </c>
-      <c r="K30" t="n">
         <v>3.896305224157907</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>[1.053536e-01, 1.479995e-01, 7.843721e-02, 1.113875e-01, 1.033692e-01, 1.093857e-01, 6.180473e-02, 9.112990e-02, 1.227403e-01, 6.839243e-02]</t>
+          <t>[1.227601e-01, 8.202800e-02, 1.282843e-01, 1.326085e-01, 1.167084e-01, 5.414252e-02, 1.291634e-01, 7.490717e-02, 1.060113e-01, 5.338633e-02]</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>0.001</v>
+        <v>0.01</v>
       </c>
       <c r="C31" t="n">
-        <v>1e-05</v>
+        <v>5000</v>
       </c>
       <c r="D31" t="n">
-        <v>1000000</v>
+        <v>0.0215605597300244</v>
       </c>
       <c r="E31" t="n">
-        <v>0.02210077568747653</v>
+        <v>0.6994625797519258</v>
       </c>
       <c r="F31" t="n">
-        <v>0.6845257047453069</v>
+        <v>0.9948626021598307</v>
       </c>
       <c r="G31" t="n">
-        <v>0.994733880812714</v>
+        <v>0.8333337542488395</v>
       </c>
       <c r="H31" t="n">
-        <v>0.8368928765702801</v>
+        <v>0.06867989045764569</v>
       </c>
       <c r="I31" t="n">
-        <v>0.06801418120635938</v>
+        <v>0.006548981438425124</v>
       </c>
       <c r="J31" t="n">
-        <v>0.006251599339498526</v>
-      </c>
-      <c r="K31" t="n">
         <v>3.896305224157907</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>[1.223005e-01, 7.574231e-02, 9.532612e-02, 8.325243e-02, 1.114118e-01, 7.322573e-02, 7.248127e-02, 1.231177e-01, 1.325967e-01, 1.105454e-01]</t>
+          <t>[7.534380e-02, 6.951502e-02, 1.318850e-01, 9.660478e-02, 6.131115e-02, 6.364028e-02, 1.414665e-01, 1.222845e-01, 9.552944e-02, 1.424195e-01]</t>
         </is>
       </c>
       <c r="B32" t="n">
         <v>0.001</v>
       </c>
       <c r="C32" t="n">
-        <v>0.01</v>
+        <v>500000</v>
       </c>
       <c r="D32" t="n">
-        <v>500000</v>
+        <v>0.03236722260145086</v>
       </c>
       <c r="E32" t="n">
-        <v>0.03068132934066005</v>
+        <v>0.6716246864116996</v>
       </c>
       <c r="F32" t="n">
-        <v>0.6718236699923352</v>
+        <v>0.9922876167610151</v>
       </c>
       <c r="G32" t="n">
-        <v>0.9926893273151562</v>
+        <v>0.8399668999051551</v>
       </c>
       <c r="H32" t="n">
-        <v>0.8399194865805388</v>
+        <v>0.06876899367401526</v>
       </c>
       <c r="I32" t="n">
-        <v>0.0683935106013917</v>
+        <v>0.00600351051621824</v>
       </c>
       <c r="J32" t="n">
-        <v>0.01220056637673716</v>
-      </c>
-      <c r="K32" t="n">
         <v>3.896305224157907</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>[1.201492e-01, 1.016427e-01, 1.422175e-01, 1.226850e-01, 8.029734e-02, 5.950230e-02, 1.334997e-01, 6.124777e-02, 6.479927e-02, 1.139592e-01]</t>
+          <t>[9.289369e-02, 7.011276e-02, 1.204170e-01, 1.235979e-01, 7.215093e-02, 9.032372e-02, 1.388188e-01, 1.402783e-01, 8.246410e-02, 6.894277e-02]</t>
         </is>
       </c>
       <c r="B33" t="n">
         <v>0.001</v>
       </c>
       <c r="C33" t="n">
-        <v>0.01</v>
+        <v>5000000</v>
       </c>
       <c r="D33" t="n">
-        <v>5000000</v>
+        <v>0.02596307154627297</v>
       </c>
       <c r="E33" t="n">
-        <v>0.02270023348454602</v>
+        <v>0.6793598473862297</v>
       </c>
       <c r="F33" t="n">
-        <v>0.6973493451517856</v>
+        <v>0.9938135823301358</v>
       </c>
       <c r="G33" t="n">
-        <v>0.9945910434638463</v>
+        <v>0.8381237845231098</v>
       </c>
       <c r="H33" t="n">
-        <v>0.8338372906600678</v>
+        <v>0.06793947348271806</v>
       </c>
       <c r="I33" t="n">
-        <v>0.0685838912101103</v>
+        <v>0.005561022010805443</v>
       </c>
       <c r="J33" t="n">
-        <v>0.005916091028005637</v>
-      </c>
-      <c r="K33" t="n">
         <v>3.896305224157907</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>[7.014742e-02, 1.508330e-01, 1.091262e-01, 7.476163e-02, 8.248312e-02, 9.601939e-02, 1.561239e-01, 9.742251e-02, 7.264423e-02, 9.043845e-02]</t>
+          <t>[6.668898e-02, 6.771992e-02, 1.383063e-01, 1.344746e-01, 9.921192e-02, 9.576794e-02, 1.065523e-01, 1.106407e-01, 1.205633e-01, 6.007409e-02]</t>
         </is>
       </c>
       <c r="B34" t="n">
         <v>0.001</v>
       </c>
       <c r="C34" t="n">
-        <v>0.01</v>
+        <v>1000000</v>
       </c>
       <c r="D34" t="n">
-        <v>1000000</v>
+        <v>0.02565739969038921</v>
       </c>
       <c r="E34" t="n">
-        <v>0.02309954353475598</v>
+        <v>0.6786253667140745</v>
       </c>
       <c r="F34" t="n">
-        <v>0.6920283769136597</v>
+        <v>0.9938864170780218</v>
       </c>
       <c r="G34" t="n">
-        <v>0.9944958968342972</v>
+        <v>0.8382987947949221</v>
       </c>
       <c r="H34" t="n">
-        <v>0.8351051580566684</v>
+        <v>0.06821713219040666</v>
       </c>
       <c r="I34" t="n">
-        <v>0.06824245252312036</v>
+        <v>-0.003469448552723169</v>
       </c>
       <c r="J34" t="n">
-        <v>0.001893168374761809</v>
-      </c>
-      <c r="K34" t="n">
         <v>3.896305224157907</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>[1.363147e-01, 1.069668e-01, 1.077072e-01, 1.370496e-01, 7.953880e-02, 5.809112e-02, 7.599820e-02, 1.543708e-01, 6.101449e-02, 8.294829e-02]</t>
+          <t>[8.450884e-02, 7.509522e-02, 7.319581e-02, 9.694183e-02, 1.478793e-01, 1.294411e-01, 1.397935e-01, 6.266517e-02, 1.119023e-01, 7.857705e-02]</t>
         </is>
       </c>
       <c r="B35" t="n">
         <v>0.001</v>
       </c>
       <c r="C35" t="n">
-        <v>0.001</v>
+        <v>100</v>
       </c>
       <c r="D35" t="n">
-        <v>500000</v>
+        <v>0.02150855880854903</v>
       </c>
       <c r="E35" t="n">
-        <v>0.02516577130838919</v>
+        <v>0.6857749211698416</v>
       </c>
       <c r="F35" t="n">
-        <v>0.6863573579044944</v>
+        <v>0.9948749928131819</v>
       </c>
       <c r="G35" t="n">
-        <v>0.9940035610955927</v>
+        <v>0.8365952163127697</v>
       </c>
       <c r="H35" t="n">
-        <v>0.8364564347013408</v>
+        <v>0.06835868109471467</v>
       </c>
       <c r="I35" t="n">
-        <v>0.06843565017118966</v>
+        <v>0.002380277732392382</v>
       </c>
       <c r="J35" t="n">
-        <v>0.01295263380961716</v>
-      </c>
-      <c r="K35" t="n">
         <v>3.896305224157907</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>[1.165246e-01, 7.349355e-02, 1.307614e-01, 1.128035e-01, 1.082670e-01, 5.976315e-02, 9.935296e-02, 6.148338e-02, 1.199135e-01, 1.176369e-01]</t>
+          <t>[1.296706e-01, 1.365847e-01, 9.724630e-02, 1.357011e-01, 6.198431e-02, 6.830490e-02, 8.286169e-02, 1.444627e-01, 5.793986e-02, 8.524383e-02]</t>
         </is>
       </c>
       <c r="B36" t="n">
         <v>0.001</v>
       </c>
       <c r="C36" t="n">
-        <v>0.001</v>
+        <v>5000</v>
       </c>
       <c r="D36" t="n">
-        <v>5000000</v>
+        <v>0.02384726596055333</v>
       </c>
       <c r="E36" t="n">
-        <v>0.02613414586410181</v>
+        <v>0.6884296591550113</v>
       </c>
       <c r="F36" t="n">
-        <v>0.6846756593787784</v>
+        <v>0.9943177313495677</v>
       </c>
       <c r="G36" t="n">
-        <v>0.9937728191569192</v>
+        <v>0.8359626517893063</v>
       </c>
       <c r="H36" t="n">
-        <v>0.83685714574419</v>
+        <v>0.06833982275699388</v>
       </c>
       <c r="I36" t="n">
-        <v>0.06819058248776809</v>
+        <v>0.01320100135284168</v>
       </c>
       <c r="J36" t="n">
-        <v>0.006329242906828085</v>
-      </c>
-      <c r="K36" t="n">
         <v>3.896305224157907</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>[1.031753e-01, 7.089498e-02, 1.009726e-01, 8.726709e-02, 1.244002e-01, 1.016202e-01, 1.560204e-01, 6.790959e-02, 1.038604e-01, 8.387927e-02]</t>
+          <t>[1.397396e-01, 9.253629e-02, 1.015469e-01, 1.314097e-01, 8.560458e-02, 8.182838e-02, 8.662082e-02, 8.903996e-02, 1.080968e-01, 8.357695e-02]</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>0.001</v>
+        <v>0.0001</v>
       </c>
       <c r="C37" t="n">
-        <v>0.001</v>
+        <v>500000</v>
       </c>
       <c r="D37" t="n">
+        <v>0.02398058424768184</v>
+      </c>
+      <c r="E37" t="n">
+        <v>0.6850767833335794</v>
+      </c>
+      <c r="F37" t="n">
+        <v>0.994285964591704</v>
+      </c>
+      <c r="G37" t="n">
+        <v>0.8367615669018575</v>
+      </c>
+      <c r="H37" t="n">
+        <v>0.06824747846120216</v>
+      </c>
+      <c r="I37" t="n">
+        <v>0.01205263217095947</v>
+      </c>
+      <c r="J37" t="n">
+        <v>3.896305224157907</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>[7.245058e-02, 7.142444e-02, 7.684398e-02, 6.490609e-02, 1.283365e-01, 8.785861e-02, 1.543154e-01, 1.209360e-01, 1.191529e-01, 1.037755e-01]</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="C38" t="n">
+        <v>5000000</v>
+      </c>
+      <c r="D38" t="n">
+        <v>0.02894302450160564</v>
+      </c>
+      <c r="E38" t="n">
+        <v>0.6748897804512357</v>
+      </c>
+      <c r="F38" t="n">
+        <v>0.9931035263729515</v>
+      </c>
+      <c r="G38" t="n">
+        <v>0.8391889012225279</v>
+      </c>
+      <c r="H38" t="n">
+        <v>0.0683275589697544</v>
+      </c>
+      <c r="I38" t="n">
+        <v>0.007656290326229435</v>
+      </c>
+      <c r="J38" t="n">
+        <v>3.896305224157907</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>[6.616910e-02, 1.326637e-01, 1.217371e-01, 8.517995e-02, 1.068308e-01, 6.677958e-02, 1.105333e-01, 6.380348e-02, 1.368143e-01, 1.094888e-01]</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="C39" t="n">
         <v>1000000</v>
       </c>
-      <c r="E37" t="n">
-        <v>0.02294155954124989</v>
-      </c>
-      <c r="F37" t="n">
-        <v>0.6885441454957046</v>
-      </c>
-      <c r="G37" t="n">
-        <v>0.9945335408768072</v>
-      </c>
-      <c r="H37" t="n">
-        <v>0.8359353722619298</v>
-      </c>
-      <c r="I37" t="n">
-        <v>0.06799996049867875</v>
-      </c>
-      <c r="J37" t="n">
-        <v>0.005381235616614728</v>
-      </c>
-      <c r="K37" t="n">
+      <c r="D39" t="n">
+        <v>0.02597930373517331</v>
+      </c>
+      <c r="E39" t="n">
+        <v>0.6855438827514648</v>
+      </c>
+      <c r="F39" t="n">
+        <v>0.9938097145635638</v>
+      </c>
+      <c r="G39" t="n">
+        <v>0.8366502675863186</v>
+      </c>
+      <c r="H39" t="n">
+        <v>0.06816633768396568</v>
+      </c>
+      <c r="I39" t="n">
+        <v>0.0003270460265995911</v>
+      </c>
+      <c r="J39" t="n">
+        <v>3.896305224157907</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>[9.118338e-02, 1.466881e-01, 1.378730e-01, 6.216409e-02, 1.412845e-01, 1.034402e-01, 8.767030e-02, 9.611348e-02, 5.978674e-02, 7.379620e-02]</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="C40" t="n">
+        <v>100</v>
+      </c>
+      <c r="D40" t="n">
+        <v>0.02135345541181115</v>
+      </c>
+      <c r="E40" t="n">
+        <v>0.699832360043354</v>
+      </c>
+      <c r="F40" t="n">
+        <v>0.994911950474086</v>
+      </c>
+      <c r="G40" t="n">
+        <v>0.8332456438985374</v>
+      </c>
+      <c r="H40" t="n">
+        <v>0.06870089951641779</v>
+      </c>
+      <c r="I40" t="n">
+        <v>-0.005362969946528121</v>
+      </c>
+      <c r="J40" t="n">
+        <v>3.896305224157907</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>[9.151051e-02, 8.279007e-02, 7.019803e-02, 1.665822e-01, 1.085886e-01, 7.442120e-02, 1.265344e-01, 8.033212e-02, 1.106713e-01, 8.837153e-02]</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="C41" t="n">
+        <v>5000</v>
+      </c>
+      <c r="D41" t="n">
+        <v>0.02170049416237909</v>
+      </c>
+      <c r="E41" t="n">
+        <v>0.6851341106168476</v>
+      </c>
+      <c r="F41" t="n">
+        <v>0.9948292589229414</v>
+      </c>
+      <c r="G41" t="n">
+        <v>0.8367479070959465</v>
+      </c>
+      <c r="H41" t="n">
+        <v>0.0682087516328107</v>
+      </c>
+      <c r="I41" t="n">
+        <v>0.009398999769031451</v>
+      </c>
+      <c r="J41" t="n">
         <v>3.896305224157907</v>
       </c>
     </row>

</xml_diff>